<commit_message>
Update Tiingo updater to use vendor_symbol on updates
</commit_message>
<xml_diff>
--- a/outputs/bucket_spreads_2025-11-05.xlsx
+++ b/outputs/bucket_spreads_2025-11-05.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="vertical_software_vs_semi_cap" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="healthcare_tools_vs_card_networks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="merchant_acquirers_vs_info_services" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -488,4 +490,146 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>avg_price_a</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>avg_price_b</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>r_1d</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>r_20d</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>r_60d</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>r_252d</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>rolling_mean</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>rolling_std</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>z_20v252</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>avg_price_a</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>avg_price_b</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>r_1d</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>r_20d</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>r_60d</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>r_252d</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>rolling_mean</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>rolling_std</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>z_20v252</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>